<commit_message>
[BUGFIX] fix Price Announcement
</commit_message>
<xml_diff>
--- a/packages/workflow/components/global/formWidget/priceAnnouncement/PriceAnnouncement_Upload_Template.xlsx
+++ b/packages/workflow/components/global/formWidget/priceAnnouncement/PriceAnnouncement_Upload_Template.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FA18B48-5493-4318-8D0F-6E414D298F07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FDB9F16-72D5-48A9-823F-17F5E9A56035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4005" yWindow="4425" windowWidth="21630" windowHeight="10155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3180" yWindow="1275" windowWidth="23085" windowHeight="11415" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="179021"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -20,7 +20,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="14">
+  <si>
+    <t>EffectiveDate</t>
+  </si>
   <si>
     <t>Index</t>
   </si>
@@ -40,17 +43,32 @@
     <t>New Unit Price</t>
   </si>
   <si>
+    <t>USD</t>
+  </si>
+  <si>
     <t>Price Group</t>
   </si>
   <si>
-    <t>EffectiveDate(yyyymmdd)</t>
+    <t>BSRSCN J</t>
+  </si>
+  <si>
+    <t>BYD</t>
+  </si>
+  <si>
+    <t>STD PRICE</t>
+  </si>
+  <si>
+    <t>RN412ESTTE F50</t>
+  </si>
+  <si>
+    <t>RN412ESTTE 8662F50</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -60,6 +78,13 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -84,14 +109,23 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="百分比" xfId="1" builtinId="5"/>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -370,44 +404,175 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="4" max="4" width="22.140625" customWidth="1"/>
     <col min="5" max="5" width="12.42578125" customWidth="1"/>
     <col min="6" max="6" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4">
+        <v>20260901</v>
+      </c>
+      <c r="C1" s="2"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4">
         <v>1</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="1" t="s">
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4">
+        <v>0.04</v>
+      </c>
+      <c r="G4">
+        <v>0.5</v>
+      </c>
+      <c r="I4" s="3"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5">
         <v>2</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5">
+        <v>0.02</v>
+      </c>
+      <c r="G5">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6">
         <v>3</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6">
+        <v>0.06</v>
+      </c>
+      <c r="G6">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7">
         <v>4</v>
       </c>
-      <c r="G3" s="1" t="s">
-        <v>5</v>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F7">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="G7">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8">
+        <v>0.06</v>
+      </c>
+      <c r="G8">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="G9">
+        <v>0.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>